<commit_message>
feat: complete B1 implementation with kit builder, end-to-end 4-Oranges order, regression tests, edge-case fixes
- Real 4-Oranges order (3 DM + 1 YCSX) with exact values and logo
- OPP sample + Tân Châu regression verified
- Kit sandbox: make_kit.py + dinh_muc_kit.zip
- Edge cases: colors=1, colors=6 (OPP 5-slot), single-product, flexo, missing dims
- .gitignore: *.bak backups
</commit_message>
<xml_diff>
--- a/templates/Định mức - Bao giấy (KP - in offset).xlsx
+++ b/templates/Định mức - Bao giấy (KP - in offset).xlsx
@@ -1410,7 +1410,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="9">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -1614,7 +1614,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1637,6 +1637,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -2722,7 +2728,7 @@
     <xf numFmtId="9" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="923">
+  <cellXfs count="1200">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -5476,10 +5482,841 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="19" fillId="5" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="19" fillId="5" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="22" fillId="5" borderId="63" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="171" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="19" fillId="5" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="5" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="19" fillId="5" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="19" fillId="5" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="19" fillId="5" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="5" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3" xr:uid="{1A2C0883-421E-4F3D-A421-1C398D21A826}"/>
+    <cellStyle name="Comma 2" xfId="3" ns2:uid="{1A2C0883-421E-4F3D-A421-1C398D21A826}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
@@ -6367,11 +7204,11 @@
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <ns4:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -9243,7 +10080,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
     <pageSetUpPr fitToPage="1"/>
@@ -9372,26 +10209,26 @@
         <v>4</v>
       </c>
       <c r="B5" s="341"/>
-      <c r="C5" s="342" t="str">
+      <c r="C5" s="1075" t="str">
         <f>V5</f>
         <v xml:space="preserve">NHÀ MÁY SX TINH BỘT SẮN TÂN CHÂU-CN CÔNG TY CPNS THỰC PHẨM QUẢNG NGÃI					</v>
       </c>
-      <c r="D5" s="343"/>
-      <c r="E5" s="343"/>
-      <c r="F5" s="343"/>
-      <c r="G5" s="344"/>
-      <c r="I5" s="345" t="s">
+      <c r="D5" s="1013"/>
+      <c r="E5" s="1012"/>
+      <c r="F5" s="989"/>
+      <c r="G5" s="962"/>
+      <c r="I5" s="992" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="346"/>
-      <c r="K5" s="346" t="s">
+      <c r="J5" s="999"/>
+      <c r="K5" s="1027" t="s">
         <v>6</v>
       </c>
-      <c r="L5" s="346"/>
-      <c r="M5" s="346" t="s">
+      <c r="L5" s="1047"/>
+      <c r="M5" s="1058" t="s">
         <v>7</v>
       </c>
-      <c r="N5" s="347"/>
+      <c r="N5" s="998"/>
       <c r="P5" s="348" t="s">
         <v>8</v>
       </c>
@@ -9420,26 +10257,26 @@
         <v>10</v>
       </c>
       <c r="B6" s="361"/>
-      <c r="C6" s="362" t="str">
+      <c r="C6" s="963" t="str">
         <f>X5</f>
         <v>Bao giấy 25kg AM-20 Tân Châu</v>
       </c>
-      <c r="D6" s="363"/>
-      <c r="E6" s="363"/>
-      <c r="F6" s="363"/>
-      <c r="G6" s="364"/>
-      <c r="I6" s="365" t="s">
+      <c r="D6" s="932"/>
+      <c r="E6" s="932"/>
+      <c r="F6" s="932"/>
+      <c r="G6" s="928"/>
+      <c r="I6" s="1031" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="366"/>
-      <c r="K6" s="367" t="s">
+      <c r="J6" s="972"/>
+      <c r="K6" s="990" t="s">
         <v>12</v>
       </c>
-      <c r="L6" s="367"/>
-      <c r="M6" s="368">
+      <c r="L6" s="1023"/>
+      <c r="M6" s="976">
         <v>5000</v>
       </c>
-      <c r="N6" s="369"/>
+      <c r="N6" s="1074"/>
       <c r="P6" s="370" t="s">
         <v>13</v>
       </c>
@@ -9462,26 +10299,26 @@
         <v>16</v>
       </c>
       <c r="B7" s="361"/>
-      <c r="C7" s="362" t="str">
+      <c r="C7" s="963" t="str">
         <f>W5</f>
         <v>BT1KH00563KP0004</v>
       </c>
-      <c r="D7" s="363"/>
-      <c r="E7" s="363"/>
-      <c r="F7" s="363"/>
-      <c r="G7" s="364"/>
-      <c r="I7" s="365" t="s">
+      <c r="D7" s="932"/>
+      <c r="E7" s="932"/>
+      <c r="F7" s="932"/>
+      <c r="G7" s="928"/>
+      <c r="I7" s="1020" t="s">
         <v>17</v>
       </c>
-      <c r="J7" s="366"/>
-      <c r="K7" s="367" t="s">
+      <c r="J7" s="961"/>
+      <c r="K7" s="1008" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="367"/>
-      <c r="M7" s="372">
+      <c r="L7" s="1049"/>
+      <c r="M7" s="952">
         <v>0.92</v>
       </c>
-      <c r="N7" s="373"/>
+      <c r="N7" s="986"/>
       <c r="P7" s="435"/>
       <c r="Q7" s="436"/>
       <c r="R7" s="418"/>
@@ -9496,26 +10333,26 @@
         <v>19</v>
       </c>
       <c r="B8" s="361"/>
-      <c r="C8" s="374" t="str">
+      <c r="C8" s="1024" t="str">
         <f>Y5</f>
         <v>26BA2HKH00563000029</v>
       </c>
-      <c r="D8" s="375"/>
-      <c r="E8" s="375"/>
-      <c r="F8" s="375"/>
-      <c r="G8" s="376"/>
-      <c r="I8" s="365" t="s">
+      <c r="D8" s="995"/>
+      <c r="E8" s="1006"/>
+      <c r="F8" s="926"/>
+      <c r="G8" s="1063"/>
+      <c r="I8" s="934" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="366"/>
-      <c r="K8" s="367" t="s">
+      <c r="J8" s="937"/>
+      <c r="K8" s="1053" t="s">
         <v>18</v>
       </c>
-      <c r="L8" s="367"/>
-      <c r="M8" s="377">
+      <c r="L8" s="970"/>
+      <c r="M8" s="1050">
         <v>0.5</v>
       </c>
-      <c r="N8" s="378"/>
+      <c r="N8" s="967"/>
       <c r="P8" s="437"/>
       <c r="Q8" s="438"/>
       <c r="R8" s="419"/>
@@ -9530,26 +10367,26 @@
         <v>21</v>
       </c>
       <c r="B9" s="380"/>
-      <c r="C9" s="381" t="s">
+      <c r="C9" s="983" t="s">
         <v>405</v>
       </c>
-      <c r="D9" s="382"/>
-      <c r="E9" s="382"/>
-      <c r="F9" s="382"/>
-      <c r="G9" s="383"/>
-      <c r="I9" s="365" t="s">
+      <c r="D9" s="1042"/>
+      <c r="E9" s="944"/>
+      <c r="F9" s="1056"/>
+      <c r="G9" s="981"/>
+      <c r="I9" s="1033" t="s">
         <v>22</v>
       </c>
-      <c r="J9" s="366"/>
-      <c r="K9" s="367" t="s">
+      <c r="J9" s="1069"/>
+      <c r="K9" s="1054" t="s">
         <v>18</v>
       </c>
-      <c r="L9" s="367"/>
-      <c r="M9" s="368">
+      <c r="L9" s="996"/>
+      <c r="M9" s="923">
         <f>M6*M7</f>
         <v>4600</v>
       </c>
-      <c r="N9" s="369"/>
+      <c r="N9" s="978"/>
       <c r="P9" s="405" t="s">
         <v>358</v>
       </c>
@@ -9571,18 +10408,18 @@
       <c r="E10" s="93"/>
       <c r="F10" s="93"/>
       <c r="G10" s="93"/>
-      <c r="I10" s="384" t="s">
+      <c r="I10" s="1077" t="s">
         <v>24</v>
       </c>
-      <c r="J10" s="385"/>
-      <c r="K10" s="368" t="s">
+      <c r="J10" s="975"/>
+      <c r="K10" s="935" t="s">
         <v>25</v>
       </c>
-      <c r="L10" s="386"/>
-      <c r="M10" s="368">
+      <c r="L10" s="1037"/>
+      <c r="M10" s="993">
         <v>2</v>
       </c>
-      <c r="N10" s="369"/>
+      <c r="N10" s="979"/>
       <c r="U10" s="111"/>
       <c r="V10" s="111"/>
       <c r="W10" s="111"/>
@@ -9595,19 +10432,19 @@
       <c r="E11" s="107"/>
       <c r="F11" s="107"/>
       <c r="G11" s="107"/>
-      <c r="I11" s="365" t="s">
+      <c r="I11" s="965" t="s">
         <v>26</v>
       </c>
-      <c r="J11" s="366"/>
-      <c r="K11" s="367" t="s">
+      <c r="J11" s="1000"/>
+      <c r="K11" s="939" t="s">
         <v>18</v>
       </c>
-      <c r="L11" s="367"/>
-      <c r="M11" s="372">
+      <c r="L11" s="982"/>
+      <c r="M11" s="950">
         <f>M8*2+0.06</f>
         <v>1.06</v>
       </c>
-      <c r="N11" s="373"/>
+      <c r="N11" s="1002"/>
       <c r="U11" s="111"/>
       <c r="V11" s="111"/>
       <c r="W11" s="111"/>
@@ -9620,16 +10457,16 @@
       <c r="E12" s="107"/>
       <c r="F12" s="107"/>
       <c r="G12" s="107"/>
-      <c r="I12" s="365" t="s">
+      <c r="I12" s="1073" t="s">
         <v>27</v>
       </c>
-      <c r="J12" s="366"/>
-      <c r="K12" s="367" t="s">
+      <c r="J12" s="1038"/>
+      <c r="K12" s="942" t="s">
         <v>18</v>
       </c>
-      <c r="L12" s="367"/>
-      <c r="M12" s="372"/>
-      <c r="N12" s="373"/>
+      <c r="L12" s="1007"/>
+      <c r="M12" s="1036"/>
+      <c r="N12" s="1004"/>
       <c r="P12" s="118"/>
       <c r="U12" s="111"/>
       <c r="V12" s="111"/>
@@ -9643,18 +10480,18 @@
       <c r="E13" s="107"/>
       <c r="F13" s="107"/>
       <c r="G13" s="107"/>
-      <c r="I13" s="365" t="s">
+      <c r="I13" s="1029" t="s">
         <v>28</v>
       </c>
-      <c r="J13" s="366"/>
-      <c r="K13" s="367" t="s">
+      <c r="J13" s="980"/>
+      <c r="K13" s="1026" t="s">
         <v>18</v>
       </c>
-      <c r="L13" s="367"/>
-      <c r="M13" s="372">
+      <c r="L13" s="968"/>
+      <c r="M13" s="958">
         <v>1.02</v>
       </c>
-      <c r="N13" s="373"/>
+      <c r="N13" s="1060"/>
       <c r="U13" s="111"/>
       <c r="V13" s="111"/>
       <c r="W13" s="111"/>
@@ -9667,19 +10504,19 @@
       <c r="E14" s="107"/>
       <c r="F14" s="107"/>
       <c r="G14" s="107"/>
-      <c r="I14" s="387" t="s">
+      <c r="I14" s="1072" t="s">
         <v>29</v>
       </c>
-      <c r="J14" s="388"/>
-      <c r="K14" s="389" t="s">
+      <c r="J14" s="1030"/>
+      <c r="K14" s="1071" t="s">
         <v>30</v>
       </c>
-      <c r="L14" s="389"/>
-      <c r="M14" s="390">
+      <c r="L14" s="1025"/>
+      <c r="M14" s="1010">
         <f>41/1000</f>
         <v>4.1000000000000002E-2</v>
       </c>
-      <c r="N14" s="391"/>
+      <c r="N14" s="933"/>
       <c r="U14" s="111"/>
       <c r="V14" s="111"/>
       <c r="W14" s="111"/>
@@ -9796,23 +10633,23 @@
       <c r="T17" s="429"/>
     </row>
     <row r="18" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A18" s="345" t="s">
+      <c r="A18" s="974" t="s">
         <v>48</v>
       </c>
-      <c r="B18" s="346">
+      <c r="B18" s="984">
         <v>1</v>
       </c>
-      <c r="C18" s="407" t="s">
+      <c r="C18" s="936" t="s">
         <v>49</v>
       </c>
-      <c r="D18" s="409" t="s">
+      <c r="D18" s="1040" t="s">
         <v>50</v>
       </c>
-      <c r="E18" s="322"/>
-      <c r="F18" s="121" t="s">
+      <c r="E18" s="1061"/>
+      <c r="F18" s="1068" t="s">
         <v>51</v>
       </c>
-      <c r="G18" s="122">
+      <c r="G18" s="1076">
         <f>M9*M13*0.07</f>
         <v>328.44000000000005</v>
       </c>
@@ -9841,15 +10678,15 @@
       </c>
     </row>
     <row r="19" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A19" s="370"/>
-      <c r="B19" s="371"/>
-      <c r="C19" s="408"/>
-      <c r="D19" s="410"/>
-      <c r="E19" s="323"/>
-      <c r="F19" s="129" t="s">
+      <c r="A19" s="947"/>
+      <c r="B19" s="940"/>
+      <c r="C19" s="1003"/>
+      <c r="D19" s="1070"/>
+      <c r="E19" s="1005"/>
+      <c r="F19" s="1039" t="s">
         <v>55</v>
       </c>
-      <c r="G19" s="130">
+      <c r="G19" s="943">
         <f>M9</f>
         <v>4600</v>
       </c>
@@ -9874,21 +10711,21 @@
       </c>
     </row>
     <row r="20" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A20" s="370"/>
-      <c r="B20" s="114">
+      <c r="A20" s="969"/>
+      <c r="B20" s="945">
         <v>2</v>
       </c>
-      <c r="C20" s="307" t="s">
+      <c r="C20" s="938" t="s">
         <v>395</v>
       </c>
-      <c r="D20" s="326" t="s">
+      <c r="D20" s="1018" t="s">
         <v>392</v>
       </c>
-      <c r="E20" s="325"/>
-      <c r="F20" s="325" t="s">
+      <c r="E20" s="1057"/>
+      <c r="F20" s="941" t="s">
         <v>51</v>
       </c>
-      <c r="G20" s="307">
+      <c r="G20" s="924">
         <v>8</v>
       </c>
       <c r="H20" s="139"/>
@@ -9912,21 +10749,21 @@
       </c>
     </row>
     <row r="21" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A21" s="370"/>
-      <c r="B21" s="114">
+      <c r="A21" s="1044"/>
+      <c r="B21" s="953">
         <v>3</v>
       </c>
-      <c r="C21" s="307" t="s">
+      <c r="C21" s="1022" t="s">
         <v>396</v>
       </c>
-      <c r="D21" s="147" t="s">
+      <c r="D21" s="927" t="s">
         <v>394</v>
       </c>
-      <c r="E21" s="137"/>
-      <c r="F21" s="316" t="s">
+      <c r="E21" s="1045"/>
+      <c r="F21" s="1009" t="s">
         <v>51</v>
       </c>
-      <c r="G21" s="138">
+      <c r="G21" s="1001">
         <v>8</v>
       </c>
       <c r="H21" s="144"/>
@@ -9954,21 +10791,21 @@
       <c r="AA21" s="145"/>
     </row>
     <row r="22" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A22" s="370"/>
-      <c r="B22" s="114">
+      <c r="A22" s="955"/>
+      <c r="B22" s="985">
         <v>4</v>
       </c>
-      <c r="C22" s="137" t="s">
+      <c r="C22" s="1046" t="s">
         <v>363</v>
       </c>
-      <c r="D22" s="137" t="s">
+      <c r="D22" s="1011" t="s">
         <v>364</v>
       </c>
-      <c r="E22" s="137"/>
-      <c r="F22" s="316" t="s">
+      <c r="E22" s="1066"/>
+      <c r="F22" s="1064" t="s">
         <v>51</v>
       </c>
-      <c r="G22" s="143">
+      <c r="G22" s="1019">
         <v>8</v>
       </c>
       <c r="H22" s="144"/>
@@ -9996,21 +10833,21 @@
       <c r="AA22" s="145"/>
     </row>
     <row r="23" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A23" s="370"/>
-      <c r="B23" s="114">
+      <c r="A23" s="956"/>
+      <c r="B23" s="1048">
         <v>5</v>
       </c>
-      <c r="C23" s="146" t="s">
+      <c r="C23" s="929" t="s">
         <v>397</v>
       </c>
-      <c r="D23" s="147" t="s">
+      <c r="D23" s="927" t="s">
         <v>398</v>
       </c>
-      <c r="E23" s="147"/>
-      <c r="F23" s="316" t="s">
+      <c r="E23" s="927"/>
+      <c r="F23" s="930" t="s">
         <v>51</v>
       </c>
-      <c r="G23" s="138"/>
+      <c r="G23" s="977"/>
       <c r="H23" s="144"/>
       <c r="I23" s="114"/>
       <c r="J23" s="114"/>
@@ -10036,15 +10873,15 @@
       <c r="AA23" s="145"/>
     </row>
     <row r="24" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A24" s="370"/>
-      <c r="B24" s="114">
+      <c r="A24" s="925"/>
+      <c r="B24" s="931">
         <v>6</v>
       </c>
-      <c r="C24" s="148"/>
-      <c r="D24" s="104"/>
-      <c r="E24" s="104"/>
-      <c r="F24" s="149"/>
-      <c r="G24" s="150"/>
+      <c r="C24" s="988"/>
+      <c r="D24" s="1078"/>
+      <c r="E24" s="991"/>
+      <c r="F24" s="997"/>
+      <c r="G24" s="1028"/>
       <c r="H24" s="144"/>
       <c r="I24" s="114"/>
       <c r="J24" s="114"/>
@@ -10070,15 +10907,15 @@
       <c r="AA24" s="145"/>
     </row>
     <row r="25" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A25" s="370"/>
-      <c r="B25" s="114">
+      <c r="A25" s="948"/>
+      <c r="B25" s="949">
         <v>7</v>
       </c>
-      <c r="C25" s="148"/>
-      <c r="D25" s="104"/>
-      <c r="E25" s="104"/>
-      <c r="F25" s="149"/>
-      <c r="G25" s="151"/>
+      <c r="C25" s="964"/>
+      <c r="D25" s="1043"/>
+      <c r="E25" s="946"/>
+      <c r="F25" s="1052"/>
+      <c r="G25" s="943"/>
       <c r="H25" s="144"/>
       <c r="I25" s="114"/>
       <c r="J25" s="114"/>
@@ -10104,15 +10941,15 @@
       <c r="AA25" s="145"/>
     </row>
     <row r="26" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A26" s="370"/>
-      <c r="B26" s="114">
+      <c r="A26" s="957"/>
+      <c r="B26" s="973">
         <v>8</v>
       </c>
-      <c r="C26" s="148"/>
-      <c r="D26" s="104"/>
-      <c r="E26" s="104"/>
-      <c r="F26" s="149"/>
-      <c r="G26" s="152"/>
+      <c r="C26" s="1051"/>
+      <c r="D26" s="954"/>
+      <c r="E26" s="1041"/>
+      <c r="F26" s="1015"/>
+      <c r="G26" s="951"/>
       <c r="H26" s="144"/>
       <c r="I26" s="114"/>
       <c r="J26" s="114"/>
@@ -10138,15 +10975,15 @@
       <c r="AA26" s="145"/>
     </row>
     <row r="27" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A27" s="370"/>
-      <c r="B27" s="114">
+      <c r="A27" s="1021"/>
+      <c r="B27" s="959">
         <v>9</v>
       </c>
-      <c r="C27" s="148"/>
-      <c r="D27" s="104"/>
-      <c r="E27" s="104"/>
-      <c r="F27" s="149"/>
-      <c r="G27" s="152"/>
+      <c r="C27" s="1065"/>
+      <c r="D27" s="1059"/>
+      <c r="E27" s="1014"/>
+      <c r="F27" s="1016"/>
+      <c r="G27" s="951"/>
       <c r="H27" s="153"/>
       <c r="I27" s="154"/>
       <c r="J27" s="154"/>
@@ -10172,15 +11009,15 @@
       <c r="AA27" s="145"/>
     </row>
     <row r="28" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A28" s="405"/>
-      <c r="B28" s="116">
+      <c r="A28" s="1032"/>
+      <c r="B28" s="1035">
         <v>10</v>
       </c>
-      <c r="C28" s="159"/>
-      <c r="D28" s="160"/>
-      <c r="E28" s="160"/>
-      <c r="F28" s="161"/>
-      <c r="G28" s="162"/>
+      <c r="C28" s="987"/>
+      <c r="D28" s="966"/>
+      <c r="E28" s="966"/>
+      <c r="F28" s="994"/>
+      <c r="G28" s="971"/>
       <c r="H28" s="163"/>
       <c r="I28" s="116"/>
       <c r="J28" s="116"/>
@@ -10206,17 +11043,17 @@
       <c r="AA28" s="145"/>
     </row>
     <row r="29" spans="1:27" ht="27.45" customHeight="1">
-      <c r="A29" s="395" t="s">
+      <c r="A29" s="1067" t="s">
         <v>75</v>
       </c>
-      <c r="B29" s="396"/>
-      <c r="C29" s="396"/>
-      <c r="D29" s="168"/>
-      <c r="E29" s="168"/>
-      <c r="F29" s="169" t="s">
+      <c r="B29" s="1034"/>
+      <c r="C29" s="1062"/>
+      <c r="D29" s="960"/>
+      <c r="E29" s="960"/>
+      <c r="F29" s="1055" t="s">
         <v>76</v>
       </c>
-      <c r="G29" s="170">
+      <c r="G29" s="1017">
         <f>M6*1.05</f>
         <v>5250</v>
       </c>
@@ -11413,7 +12250,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
     <pageSetUpPr fitToPage="1"/>
@@ -11501,15 +12338,15 @@
       <c r="A5" s="92" t="s">
         <v>116</v>
       </c>
-      <c r="C5" s="575" t="str">
+      <c r="C5" s="1121" t="str">
         <f>In!C8</f>
         <v>26BA2HKH00563000029</v>
       </c>
-      <c r="D5" s="575"/>
-      <c r="E5" s="93"/>
-      <c r="F5" s="93"/>
-      <c r="G5" s="93"/>
-      <c r="H5" s="93"/>
+      <c r="D5" s="1094"/>
+      <c r="E5" s="1093"/>
+      <c r="F5" s="1113"/>
+      <c r="G5" s="1082"/>
+      <c r="H5" s="1083"/>
       <c r="I5" s="92" t="s">
         <v>3</v>
       </c>
@@ -11522,15 +12359,15 @@
       <c r="A6" s="92" t="s">
         <v>117</v>
       </c>
-      <c r="C6" s="642" t="str">
+      <c r="C6" s="1084" t="str">
         <f>In!C7</f>
         <v>BT1KH00563KP0004</v>
       </c>
-      <c r="D6" s="642"/>
-      <c r="E6" s="95"/>
-      <c r="F6" s="95"/>
-      <c r="G6" s="95"/>
-      <c r="H6" s="93"/>
+      <c r="D6" s="1084"/>
+      <c r="E6" s="1084"/>
+      <c r="F6" s="1084"/>
+      <c r="G6" s="1084"/>
+      <c r="H6" s="1098"/>
       <c r="I6" s="92" t="s">
         <v>118</v>
       </c>
@@ -11542,15 +12379,15 @@
       <c r="A7" s="92" t="s">
         <v>120</v>
       </c>
-      <c r="C7" s="575" t="str">
+      <c r="C7" s="1117" t="str">
         <f>In!C6</f>
         <v>Bao giấy 25kg AM-20 Tân Châu</v>
       </c>
-      <c r="D7" s="575"/>
-      <c r="E7" s="575"/>
-      <c r="F7" s="575"/>
-      <c r="G7" s="575"/>
-      <c r="H7" s="575"/>
+      <c r="D7" s="1105"/>
+      <c r="E7" s="1087"/>
+      <c r="F7" s="1120"/>
+      <c r="G7" s="1095"/>
+      <c r="H7" s="1085"/>
       <c r="I7" s="92" t="s">
         <v>121</v>
       </c>
@@ -11563,15 +12400,15 @@
         <v>123</v>
       </c>
       <c r="B8" s="94"/>
-      <c r="C8" s="575" t="str">
+      <c r="C8" s="1108" t="str">
         <f>In!C5</f>
         <v xml:space="preserve">NHÀ MÁY SX TINH BỘT SẮN TÂN CHÂU-CN CÔNG TY CPNS THỰC PHẨM QUẢNG NGÃI					</v>
       </c>
-      <c r="D8" s="575"/>
-      <c r="E8" s="575"/>
-      <c r="F8" s="575"/>
-      <c r="G8" s="575"/>
-      <c r="H8" s="575"/>
+      <c r="D8" s="1119"/>
+      <c r="E8" s="1086"/>
+      <c r="F8" s="1081"/>
+      <c r="G8" s="1109"/>
+      <c r="H8" s="1088"/>
       <c r="I8" s="92" t="s">
         <v>124</v>
       </c>
@@ -11694,14 +12531,14 @@
         <v>135</v>
       </c>
       <c r="B16" s="653"/>
-      <c r="C16" s="441" t="str">
+      <c r="C16" s="1097" t="str">
         <f>'In 1'!C16</f>
         <v>Bao KP</v>
       </c>
-      <c r="D16" s="441"/>
-      <c r="E16" s="441"/>
-      <c r="F16" s="441"/>
-      <c r="G16" s="453"/>
+      <c r="D16" s="1106"/>
+      <c r="E16" s="1089"/>
+      <c r="F16" s="1096"/>
+      <c r="G16" s="1090"/>
       <c r="I16" s="643" t="s">
         <v>137</v>
       </c>
@@ -11716,16 +12553,16 @@
         <v>139</v>
       </c>
       <c r="B17" s="653"/>
-      <c r="C17" s="654" t="str">
+      <c r="C17" s="1110" t="str">
         <f>'In 1'!C17</f>
         <v>500 x 920</v>
       </c>
-      <c r="D17" s="654"/>
-      <c r="E17" s="654"/>
-      <c r="F17" s="371" t="s">
+      <c r="D17" s="1112"/>
+      <c r="E17" s="1091"/>
+      <c r="F17" s="1111" t="s">
         <v>140</v>
       </c>
-      <c r="G17" s="646"/>
+      <c r="G17" s="1092"/>
       <c r="I17" s="612"/>
       <c r="J17" s="613"/>
       <c r="K17" s="615"/>
@@ -11736,16 +12573,16 @@
         <v>141</v>
       </c>
       <c r="B18" s="653"/>
-      <c r="C18" s="654" t="str">
+      <c r="C18" s="1099" t="str">
         <f>'In 1'!C18</f>
         <v>500 x 920</v>
       </c>
-      <c r="D18" s="654"/>
-      <c r="E18" s="654"/>
-      <c r="F18" s="371" t="s">
+      <c r="D18" s="1118"/>
+      <c r="E18" s="1104"/>
+      <c r="F18" s="1114" t="s">
         <v>140</v>
       </c>
-      <c r="G18" s="646"/>
+      <c r="G18" s="1122"/>
       <c r="I18" s="612"/>
       <c r="J18" s="613"/>
       <c r="K18" s="615"/>
@@ -11756,16 +12593,16 @@
         <v>142</v>
       </c>
       <c r="B19" s="653"/>
-      <c r="C19" s="654">
+      <c r="C19" s="1123">
         <f>In!M6</f>
         <v>5000</v>
       </c>
-      <c r="D19" s="654"/>
-      <c r="E19" s="654"/>
-      <c r="F19" s="371" t="s">
+      <c r="D19" s="1116"/>
+      <c r="E19" s="1080"/>
+      <c r="F19" s="1115" t="s">
         <v>12</v>
       </c>
-      <c r="G19" s="646"/>
+      <c r="G19" s="1107"/>
       <c r="I19" s="612"/>
       <c r="J19" s="613"/>
       <c r="K19" s="615"/>
@@ -11776,16 +12613,16 @@
         <v>143</v>
       </c>
       <c r="B20" s="656"/>
-      <c r="C20" s="657">
+      <c r="C20" s="1101">
         <f>C19</f>
         <v>5000</v>
       </c>
-      <c r="D20" s="657"/>
-      <c r="E20" s="657"/>
-      <c r="F20" s="439" t="s">
+      <c r="D20" s="1100"/>
+      <c r="E20" s="1102"/>
+      <c r="F20" s="1103" t="s">
         <v>12</v>
       </c>
-      <c r="G20" s="658"/>
+      <c r="G20" s="1079"/>
       <c r="I20" s="647"/>
       <c r="J20" s="648"/>
       <c r="K20" s="650"/>
@@ -17033,7 +17870,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-1100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
     <pageSetUpPr fitToPage="1"/>
@@ -17145,15 +17982,15 @@
         <v>116</v>
       </c>
       <c r="B5" s="767"/>
-      <c r="C5" s="768" t="str">
+      <c r="C5" s="1150" t="str">
         <f>'In 2'!C5</f>
         <v>26BA2HKH00563000029</v>
       </c>
-      <c r="D5" s="768"/>
-      <c r="E5" s="768"/>
-      <c r="F5" s="768"/>
-      <c r="G5" s="768"/>
-      <c r="H5" s="768"/>
+      <c r="D5" s="1136"/>
+      <c r="E5" s="1135"/>
+      <c r="F5" s="1146"/>
+      <c r="G5" s="1125"/>
+      <c r="H5" s="1126"/>
       <c r="I5" s="48" t="s">
         <v>3</v>
       </c>
@@ -17188,15 +18025,15 @@
         <v>117</v>
       </c>
       <c r="B6" s="769"/>
-      <c r="C6" s="770" t="str">
+      <c r="C6" s="1127" t="str">
         <f>'In 2'!C6</f>
         <v>BT1KH00563KP0004</v>
       </c>
-      <c r="D6" s="770"/>
-      <c r="E6" s="770"/>
-      <c r="F6" s="770"/>
-      <c r="G6" s="770"/>
-      <c r="H6" s="770"/>
+      <c r="D6" s="1137"/>
+      <c r="E6" s="1128"/>
+      <c r="F6" s="1151"/>
+      <c r="G6" s="1129"/>
+      <c r="H6" s="1140"/>
       <c r="I6" s="48" t="s">
         <v>184</v>
       </c>
@@ -17215,15 +18052,15 @@
         <v>120</v>
       </c>
       <c r="B7" s="769"/>
-      <c r="C7" s="770" t="str">
+      <c r="C7" s="1147" t="str">
         <f>'In 2'!C7</f>
         <v>Bao giấy 25kg AM-20 Tân Châu</v>
       </c>
-      <c r="D7" s="770"/>
-      <c r="E7" s="770"/>
-      <c r="F7" s="770"/>
-      <c r="G7" s="770"/>
-      <c r="H7" s="770"/>
+      <c r="D7" s="1141"/>
+      <c r="E7" s="1132"/>
+      <c r="F7" s="1149"/>
+      <c r="G7" s="1138"/>
+      <c r="H7" s="1130"/>
       <c r="I7" s="5" t="s">
         <v>121</v>
       </c>
@@ -17243,15 +18080,15 @@
         <v>123</v>
       </c>
       <c r="B8" s="769"/>
-      <c r="C8" s="768" t="str">
+      <c r="C8" s="1143" t="str">
         <f>'In 2'!C8</f>
         <v xml:space="preserve">NHÀ MÁY SX TINH BỘT SẮN TÂN CHÂU-CN CÔNG TY CPNS THỰC PHẨM QUẢNG NGÃI					</v>
       </c>
-      <c r="D8" s="768"/>
-      <c r="E8" s="768"/>
-      <c r="F8" s="768"/>
-      <c r="G8" s="768"/>
-      <c r="H8" s="768"/>
+      <c r="D8" s="1148"/>
+      <c r="E8" s="1131"/>
+      <c r="F8" s="1124"/>
+      <c r="G8" s="1145"/>
+      <c r="H8" s="1133"/>
       <c r="I8" s="5" t="s">
         <v>124</v>
       </c>
@@ -17423,20 +18260,20 @@
         <v>186</v>
       </c>
       <c r="B16" s="13"/>
-      <c r="C16" s="801">
+      <c r="C16" s="1139">
         <f>'In 2'!C16</f>
         <v>4600</v>
       </c>
-      <c r="D16" s="802"/>
+      <c r="D16" s="1142"/>
       <c r="E16" s="803" t="s">
         <v>187</v>
       </c>
       <c r="F16" s="803"/>
-      <c r="G16" s="804">
+      <c r="G16" s="1134">
         <f>Tráng!M9</f>
         <v>4600</v>
       </c>
-      <c r="H16" s="805"/>
+      <c r="H16" s="1144"/>
       <c r="I16" s="7"/>
       <c r="J16" s="806" t="s">
         <v>137</v>
@@ -21603,7 +22440,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-1300-000000000000}">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
     <pageSetUpPr fitToPage="1"/>
@@ -21691,15 +22528,15 @@
         <v>116</v>
       </c>
       <c r="B5" s="576"/>
-      <c r="C5" s="575" t="str">
+      <c r="C5" s="1196" t="str">
         <f>'In 2'!C5</f>
         <v>26BA2HKH00563000029</v>
       </c>
-      <c r="D5" s="575"/>
-      <c r="E5" s="575"/>
-      <c r="F5" s="575"/>
-      <c r="G5" s="575"/>
-      <c r="H5" s="575"/>
+      <c r="D5" s="1166"/>
+      <c r="E5" s="1165"/>
+      <c r="F5" s="1185"/>
+      <c r="G5" s="1155"/>
+      <c r="H5" s="1156"/>
       <c r="I5" s="92" t="s">
         <v>3</v>
       </c>
@@ -21726,15 +22563,15 @@
         <v>117</v>
       </c>
       <c r="B6" s="577"/>
-      <c r="C6" s="338" t="str">
+      <c r="C6" s="1157" t="str">
         <f>'In 2'!C6</f>
         <v>BT1KH00563KP0004</v>
       </c>
-      <c r="D6" s="338"/>
-      <c r="E6" s="338"/>
-      <c r="F6" s="338"/>
-      <c r="G6" s="338"/>
-      <c r="H6" s="338"/>
+      <c r="D6" s="1167"/>
+      <c r="E6" s="1158"/>
+      <c r="F6" s="1199"/>
+      <c r="G6" s="1159"/>
+      <c r="H6" s="1169"/>
       <c r="I6" s="92" t="s">
         <v>184</v>
       </c>
@@ -21748,15 +22585,15 @@
         <v>120</v>
       </c>
       <c r="B7" s="577"/>
-      <c r="C7" s="338" t="str">
+      <c r="C7" s="1190" t="str">
         <f>'In 2'!C7</f>
         <v>Bao giấy 25kg AM-20 Tân Châu</v>
       </c>
-      <c r="D7" s="338"/>
-      <c r="E7" s="338"/>
-      <c r="F7" s="338"/>
-      <c r="G7" s="338"/>
-      <c r="H7" s="338"/>
+      <c r="D7" s="1177"/>
+      <c r="E7" s="1162"/>
+      <c r="F7" s="1194"/>
+      <c r="G7" s="1168"/>
+      <c r="H7" s="1160"/>
       <c r="I7" s="180" t="s">
         <v>121</v>
       </c>
@@ -21770,15 +22607,15 @@
         <v>123</v>
       </c>
       <c r="B8" s="577"/>
-      <c r="C8" s="575" t="str">
+      <c r="C8" s="1180" t="str">
         <f>'In 2'!C8</f>
         <v xml:space="preserve">NHÀ MÁY SX TINH BỘT SẮN TÂN CHÂU-CN CÔNG TY CPNS THỰC PHẨM QUẢNG NGÃI					</v>
       </c>
-      <c r="D8" s="575"/>
-      <c r="E8" s="575"/>
-      <c r="F8" s="575"/>
-      <c r="G8" s="575"/>
-      <c r="H8" s="575"/>
+      <c r="D8" s="1192"/>
+      <c r="E8" s="1161"/>
+      <c r="F8" s="1154"/>
+      <c r="G8" s="1182"/>
+      <c r="H8" s="1163"/>
       <c r="I8" s="180" t="s">
         <v>124</v>
       </c>
@@ -21790,9 +22627,9 @@
     <row r="9" spans="1:24" ht="15" customHeight="1">
       <c r="A9" s="94"/>
       <c r="B9" s="94"/>
-      <c r="C9" s="94"/>
-      <c r="D9" s="94"/>
-      <c r="E9" s="94"/>
+      <c r="C9" s="1183"/>
+      <c r="D9" s="1193"/>
+      <c r="E9" s="1179"/>
       <c r="I9" s="94"/>
       <c r="K9" s="94"/>
     </row>
@@ -21948,26 +22785,26 @@
       <c r="A18" s="140">
         <v>1</v>
       </c>
-      <c r="B18" s="333">
+      <c r="B18" s="1184">
         <f>Dán!C17</f>
         <v>9415</v>
       </c>
-      <c r="C18" s="333"/>
-      <c r="D18" s="210" t="str">
+      <c r="C18" s="1170"/>
+      <c r="D18" s="1191" t="str">
         <f>Dán!D17</f>
         <v>NHPPFC9415G01</v>
       </c>
-      <c r="E18" s="188">
+      <c r="E18" s="1176">
         <v>0.6</v>
       </c>
-      <c r="F18" s="189" t="s">
+      <c r="F18" s="1186" t="s">
         <v>51</v>
       </c>
-      <c r="G18" s="189">
+      <c r="G18" s="1197">
         <f>Dán!G17</f>
         <v>9.1466399999999997</v>
       </c>
-      <c r="H18" s="186"/>
+      <c r="H18" s="1187"/>
       <c r="J18" s="672"/>
       <c r="K18" s="673"/>
       <c r="L18" s="191"/>
@@ -21977,44 +22814,44 @@
       <c r="A19" s="140">
         <v>2</v>
       </c>
-      <c r="B19" s="333" t="str">
+      <c r="B19" s="1174" t="str">
         <f>Dán!C18</f>
         <v>Vistamaxx</v>
       </c>
-      <c r="C19" s="333"/>
-      <c r="D19" s="210" t="str">
+      <c r="C19" s="1198"/>
+      <c r="D19" s="1189" t="str">
         <f>Dán!D18</f>
         <v>NHVITAMAX0001</v>
       </c>
-      <c r="E19" s="188">
+      <c r="E19" s="1153">
         <v>0.4</v>
       </c>
-      <c r="F19" s="189" t="s">
+      <c r="F19" s="1188" t="s">
         <v>51</v>
       </c>
-      <c r="G19" s="189">
+      <c r="G19" s="1178">
         <f>Dán!G18</f>
         <v>6.0977600000000001</v>
       </c>
-      <c r="H19" s="190"/>
+      <c r="H19" s="1195"/>
     </row>
     <row r="20" spans="1:14" ht="18" customHeight="1">
       <c r="A20" s="140">
         <v>3</v>
       </c>
-      <c r="B20" s="441" t="str">
+      <c r="B20" s="1181" t="str">
         <f>Dán!C19</f>
         <v>Keo Acrylic</v>
       </c>
-      <c r="C20" s="441"/>
-      <c r="D20" s="210" t="str">
+      <c r="C20" s="1172"/>
+      <c r="D20" s="1171" t="str">
         <f>Dán!D19</f>
         <v>PKACRYLIC0001</v>
       </c>
-      <c r="E20" s="188"/>
-      <c r="F20" s="114"/>
-      <c r="G20" s="189"/>
-      <c r="H20" s="190"/>
+      <c r="E20" s="1173"/>
+      <c r="F20" s="1175"/>
+      <c r="G20" s="1152"/>
+      <c r="H20" s="1164"/>
       <c r="J20" s="348" t="s">
         <v>192</v>
       </c>

</xml_diff>

<commit_message>
feat: re-derive Định mức templates from golden refs (white output, no yellow)
Templates now sourced from the golden 25kg/40kg references instead of the
boss's yellow-marked working copies. Input cells cleared byte-surgically;
golden is all-white so every output prints clean (no FFFFFF00 markers).

- OPP template  <- Định mức - 4O BTA140 40KG golden
- paper template <- Định mức - Bao giấy 25kg Tân Châu golden
- 0 yellow in both; 0 validator issues; format identical to golden (23 sheets,
  merges/widths/heights/dims all match); regression values unchanged.
- YCSX template untouched (already 0 yellow).
- kit rebuilt (13 files).

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/Định mức - Bao giấy (KP - in offset).xlsx
+++ b/templates/Định mức - Bao giấy (KP - in offset).xlsx
@@ -1410,7 +1410,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns4="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="9">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -1614,7 +1614,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1637,12 +1637,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -2728,7 +2722,7 @@
     <xf numFmtId="9" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1200">
+  <cellXfs count="923">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -5482,841 +5476,10 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="19" fillId="5" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="19" fillId="5" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="5" borderId="63" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="171" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="29" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="19" fillId="5" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="29" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="5" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="68" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="19" fillId="5" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="19" fillId="5" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="19" fillId="5" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="5" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="19" fillId="5" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyFill="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3" ns2:uid="{1A2C0883-421E-4F3D-A421-1C398D21A826}"/>
+    <cellStyle name="Comma 2" xfId="3" xr:uid="{1A2C0883-421E-4F3D-A421-1C398D21A826}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
@@ -7204,11 +6367,11 @@
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <ns4:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -10080,7 +9243,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
     <pageSetUpPr fitToPage="1"/>
@@ -10209,26 +9372,23 @@
         <v>4</v>
       </c>
       <c r="B5" s="341"/>
-      <c r="C5" s="1075" t="str">
-        <f>V5</f>
-        <v xml:space="preserve">NHÀ MÁY SX TINH BỘT SẮN TÂN CHÂU-CN CÔNG TY CPNS THỰC PHẨM QUẢNG NGÃI					</v>
-      </c>
-      <c r="D5" s="1013"/>
-      <c r="E5" s="1012"/>
-      <c r="F5" s="989"/>
-      <c r="G5" s="962"/>
-      <c r="I5" s="992" t="s">
+      <c r="C5" s="342"/>
+      <c r="D5" s="343"/>
+      <c r="E5" s="343"/>
+      <c r="F5" s="343"/>
+      <c r="G5" s="344"/>
+      <c r="I5" s="345" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="999"/>
-      <c r="K5" s="1027" t="s">
+      <c r="J5" s="346"/>
+      <c r="K5" s="346" t="s">
         <v>6</v>
       </c>
-      <c r="L5" s="1047"/>
-      <c r="M5" s="1058" t="s">
+      <c r="L5" s="346"/>
+      <c r="M5" s="346" t="s">
         <v>7</v>
       </c>
-      <c r="N5" s="998"/>
+      <c r="N5" s="347"/>
       <c r="P5" s="348" t="s">
         <v>8</v>
       </c>
@@ -10257,26 +9417,21 @@
         <v>10</v>
       </c>
       <c r="B6" s="361"/>
-      <c r="C6" s="963" t="str">
-        <f>X5</f>
-        <v>Bao giấy 25kg AM-20 Tân Châu</v>
-      </c>
-      <c r="D6" s="932"/>
-      <c r="E6" s="932"/>
-      <c r="F6" s="932"/>
-      <c r="G6" s="928"/>
-      <c r="I6" s="1031" t="s">
+      <c r="C6" s="362"/>
+      <c r="D6" s="363"/>
+      <c r="E6" s="363"/>
+      <c r="F6" s="363"/>
+      <c r="G6" s="364"/>
+      <c r="I6" s="365" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="972"/>
-      <c r="K6" s="990" t="s">
+      <c r="J6" s="366"/>
+      <c r="K6" s="367" t="s">
         <v>12</v>
       </c>
-      <c r="L6" s="1023"/>
-      <c r="M6" s="976">
-        <v>5000</v>
-      </c>
-      <c r="N6" s="1074"/>
+      <c r="L6" s="367"/>
+      <c r="M6" s="368"/>
+      <c r="N6" s="369"/>
       <c r="P6" s="370" t="s">
         <v>13</v>
       </c>
@@ -10299,26 +9454,21 @@
         <v>16</v>
       </c>
       <c r="B7" s="361"/>
-      <c r="C7" s="963" t="str">
-        <f>W5</f>
-        <v>BT1KH00563KP0004</v>
-      </c>
-      <c r="D7" s="932"/>
-      <c r="E7" s="932"/>
-      <c r="F7" s="932"/>
-      <c r="G7" s="928"/>
-      <c r="I7" s="1020" t="s">
+      <c r="C7" s="362"/>
+      <c r="D7" s="363"/>
+      <c r="E7" s="363"/>
+      <c r="F7" s="363"/>
+      <c r="G7" s="364"/>
+      <c r="I7" s="365" t="s">
         <v>17</v>
       </c>
-      <c r="J7" s="961"/>
-      <c r="K7" s="1008" t="s">
+      <c r="J7" s="366"/>
+      <c r="K7" s="367" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="1049"/>
-      <c r="M7" s="952">
-        <v>0.92</v>
-      </c>
-      <c r="N7" s="986"/>
+      <c r="L7" s="367"/>
+      <c r="M7" s="372"/>
+      <c r="N7" s="373"/>
       <c r="P7" s="435"/>
       <c r="Q7" s="436"/>
       <c r="R7" s="418"/>
@@ -10333,26 +9483,21 @@
         <v>19</v>
       </c>
       <c r="B8" s="361"/>
-      <c r="C8" s="1024" t="str">
-        <f>Y5</f>
-        <v>26BA2HKH00563000029</v>
-      </c>
-      <c r="D8" s="995"/>
-      <c r="E8" s="1006"/>
-      <c r="F8" s="926"/>
-      <c r="G8" s="1063"/>
-      <c r="I8" s="934" t="s">
+      <c r="C8" s="374"/>
+      <c r="D8" s="375"/>
+      <c r="E8" s="375"/>
+      <c r="F8" s="375"/>
+      <c r="G8" s="376"/>
+      <c r="I8" s="365" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="937"/>
-      <c r="K8" s="1053" t="s">
+      <c r="J8" s="366"/>
+      <c r="K8" s="367" t="s">
         <v>18</v>
       </c>
-      <c r="L8" s="970"/>
-      <c r="M8" s="1050">
-        <v>0.5</v>
-      </c>
-      <c r="N8" s="967"/>
+      <c r="L8" s="367"/>
+      <c r="M8" s="377"/>
+      <c r="N8" s="378"/>
       <c r="P8" s="437"/>
       <c r="Q8" s="438"/>
       <c r="R8" s="419"/>
@@ -10367,26 +9512,21 @@
         <v>21</v>
       </c>
       <c r="B9" s="380"/>
-      <c r="C9" s="983" t="s">
-        <v>405</v>
-      </c>
-      <c r="D9" s="1042"/>
-      <c r="E9" s="944"/>
-      <c r="F9" s="1056"/>
-      <c r="G9" s="981"/>
-      <c r="I9" s="1033" t="s">
+      <c r="C9" s="381"/>
+      <c r="D9" s="382"/>
+      <c r="E9" s="382"/>
+      <c r="F9" s="382"/>
+      <c r="G9" s="383"/>
+      <c r="I9" s="365" t="s">
         <v>22</v>
       </c>
-      <c r="J9" s="1069"/>
-      <c r="K9" s="1054" t="s">
+      <c r="J9" s="366"/>
+      <c r="K9" s="367" t="s">
         <v>18</v>
       </c>
-      <c r="L9" s="996"/>
-      <c r="M9" s="923">
-        <f>M6*M7</f>
-        <v>4600</v>
-      </c>
-      <c r="N9" s="978"/>
+      <c r="L9" s="367"/>
+      <c r="M9" s="368"/>
+      <c r="N9" s="369"/>
       <c r="P9" s="405" t="s">
         <v>358</v>
       </c>
@@ -10408,18 +9548,16 @@
       <c r="E10" s="93"/>
       <c r="F10" s="93"/>
       <c r="G10" s="93"/>
-      <c r="I10" s="1077" t="s">
+      <c r="I10" s="384" t="s">
         <v>24</v>
       </c>
-      <c r="J10" s="975"/>
-      <c r="K10" s="935" t="s">
+      <c r="J10" s="385"/>
+      <c r="K10" s="368" t="s">
         <v>25</v>
       </c>
-      <c r="L10" s="1037"/>
-      <c r="M10" s="993">
-        <v>2</v>
-      </c>
-      <c r="N10" s="979"/>
+      <c r="L10" s="386"/>
+      <c r="M10" s="368"/>
+      <c r="N10" s="369"/>
       <c r="U10" s="111"/>
       <c r="V10" s="111"/>
       <c r="W10" s="111"/>
@@ -10432,19 +9570,16 @@
       <c r="E11" s="107"/>
       <c r="F11" s="107"/>
       <c r="G11" s="107"/>
-      <c r="I11" s="965" t="s">
+      <c r="I11" s="365" t="s">
         <v>26</v>
       </c>
-      <c r="J11" s="1000"/>
-      <c r="K11" s="939" t="s">
+      <c r="J11" s="366"/>
+      <c r="K11" s="367" t="s">
         <v>18</v>
       </c>
-      <c r="L11" s="982"/>
-      <c r="M11" s="950">
-        <f>M8*2+0.06</f>
-        <v>1.06</v>
-      </c>
-      <c r="N11" s="1002"/>
+      <c r="L11" s="367"/>
+      <c r="M11" s="372"/>
+      <c r="N11" s="373"/>
       <c r="U11" s="111"/>
       <c r="V11" s="111"/>
       <c r="W11" s="111"/>
@@ -10457,16 +9592,16 @@
       <c r="E12" s="107"/>
       <c r="F12" s="107"/>
       <c r="G12" s="107"/>
-      <c r="I12" s="1073" t="s">
+      <c r="I12" s="365" t="s">
         <v>27</v>
       </c>
-      <c r="J12" s="1038"/>
-      <c r="K12" s="942" t="s">
+      <c r="J12" s="366"/>
+      <c r="K12" s="367" t="s">
         <v>18</v>
       </c>
-      <c r="L12" s="1007"/>
-      <c r="M12" s="1036"/>
-      <c r="N12" s="1004"/>
+      <c r="L12" s="367"/>
+      <c r="M12" s="372"/>
+      <c r="N12" s="373"/>
       <c r="P12" s="118"/>
       <c r="U12" s="111"/>
       <c r="V12" s="111"/>
@@ -10480,18 +9615,16 @@
       <c r="E13" s="107"/>
       <c r="F13" s="107"/>
       <c r="G13" s="107"/>
-      <c r="I13" s="1029" t="s">
+      <c r="I13" s="365" t="s">
         <v>28</v>
       </c>
-      <c r="J13" s="980"/>
-      <c r="K13" s="1026" t="s">
+      <c r="J13" s="366"/>
+      <c r="K13" s="367" t="s">
         <v>18</v>
       </c>
-      <c r="L13" s="968"/>
-      <c r="M13" s="958">
-        <v>1.02</v>
-      </c>
-      <c r="N13" s="1060"/>
+      <c r="L13" s="367"/>
+      <c r="M13" s="372"/>
+      <c r="N13" s="373"/>
       <c r="U13" s="111"/>
       <c r="V13" s="111"/>
       <c r="W13" s="111"/>
@@ -10504,19 +9637,16 @@
       <c r="E14" s="107"/>
       <c r="F14" s="107"/>
       <c r="G14" s="107"/>
-      <c r="I14" s="1072" t="s">
+      <c r="I14" s="387" t="s">
         <v>29</v>
       </c>
-      <c r="J14" s="1030"/>
-      <c r="K14" s="1071" t="s">
+      <c r="J14" s="388"/>
+      <c r="K14" s="389" t="s">
         <v>30</v>
       </c>
-      <c r="L14" s="1025"/>
-      <c r="M14" s="1010">
-        <f>41/1000</f>
-        <v>4.1000000000000002E-2</v>
-      </c>
-      <c r="N14" s="933"/>
+      <c r="L14" s="389"/>
+      <c r="M14" s="390"/>
+      <c r="N14" s="391"/>
       <c r="U14" s="111"/>
       <c r="V14" s="111"/>
       <c r="W14" s="111"/>
@@ -10633,26 +9763,13 @@
       <c r="T17" s="429"/>
     </row>
     <row r="18" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A18" s="974" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="984">
-        <v>1</v>
-      </c>
-      <c r="C18" s="936" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18" s="1040" t="s">
-        <v>50</v>
-      </c>
-      <c r="E18" s="1061"/>
-      <c r="F18" s="1068" t="s">
-        <v>51</v>
-      </c>
-      <c r="G18" s="1076">
-        <f>M9*M13*0.07</f>
-        <v>328.44000000000005</v>
-      </c>
+      <c r="A18" s="345"/>
+      <c r="B18" s="346"/>
+      <c r="C18" s="407"/>
+      <c r="D18" s="409"/>
+      <c r="E18" s="322"/>
+      <c r="F18" s="121"/>
+      <c r="G18" s="122"/>
       <c r="H18" s="123"/>
       <c r="I18" s="124"/>
       <c r="J18" s="124"/>
@@ -10678,18 +9795,13 @@
       </c>
     </row>
     <row r="19" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A19" s="947"/>
-      <c r="B19" s="940"/>
-      <c r="C19" s="1003"/>
-      <c r="D19" s="1070"/>
-      <c r="E19" s="1005"/>
-      <c r="F19" s="1039" t="s">
-        <v>55</v>
-      </c>
-      <c r="G19" s="943">
-        <f>M9</f>
-        <v>4600</v>
-      </c>
+      <c r="A19" s="370"/>
+      <c r="B19" s="371"/>
+      <c r="C19" s="408"/>
+      <c r="D19" s="410"/>
+      <c r="E19" s="323"/>
+      <c r="F19" s="129"/>
+      <c r="G19" s="130"/>
       <c r="H19" s="131"/>
       <c r="I19" s="132"/>
       <c r="J19" s="132"/>
@@ -10711,23 +9823,13 @@
       </c>
     </row>
     <row r="20" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A20" s="969"/>
-      <c r="B20" s="945">
-        <v>2</v>
-      </c>
-      <c r="C20" s="938" t="s">
-        <v>395</v>
-      </c>
-      <c r="D20" s="1018" t="s">
-        <v>392</v>
-      </c>
-      <c r="E20" s="1057"/>
-      <c r="F20" s="941" t="s">
-        <v>51</v>
-      </c>
-      <c r="G20" s="924">
-        <v>8</v>
-      </c>
+      <c r="A20" s="370"/>
+      <c r="B20" s="114"/>
+      <c r="C20" s="307"/>
+      <c r="D20" s="326"/>
+      <c r="E20" s="325"/>
+      <c r="F20" s="325"/>
+      <c r="G20" s="307"/>
       <c r="H20" s="139"/>
       <c r="I20" s="114"/>
       <c r="J20" s="114"/>
@@ -10749,23 +9851,13 @@
       </c>
     </row>
     <row r="21" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A21" s="1044"/>
-      <c r="B21" s="953">
-        <v>3</v>
-      </c>
-      <c r="C21" s="1022" t="s">
-        <v>396</v>
-      </c>
-      <c r="D21" s="927" t="s">
-        <v>394</v>
-      </c>
-      <c r="E21" s="1045"/>
-      <c r="F21" s="1009" t="s">
-        <v>51</v>
-      </c>
-      <c r="G21" s="1001">
-        <v>8</v>
-      </c>
+      <c r="A21" s="370"/>
+      <c r="B21" s="114"/>
+      <c r="C21" s="307"/>
+      <c r="D21" s="147"/>
+      <c r="E21" s="137"/>
+      <c r="F21" s="316"/>
+      <c r="G21" s="138"/>
       <c r="H21" s="144"/>
       <c r="I21" s="114"/>
       <c r="J21" s="114"/>
@@ -10791,23 +9883,13 @@
       <c r="AA21" s="145"/>
     </row>
     <row r="22" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A22" s="955"/>
-      <c r="B22" s="985">
-        <v>4</v>
-      </c>
-      <c r="C22" s="1046" t="s">
-        <v>363</v>
-      </c>
-      <c r="D22" s="1011" t="s">
-        <v>364</v>
-      </c>
-      <c r="E22" s="1066"/>
-      <c r="F22" s="1064" t="s">
-        <v>51</v>
-      </c>
-      <c r="G22" s="1019">
-        <v>8</v>
-      </c>
+      <c r="A22" s="370"/>
+      <c r="B22" s="114"/>
+      <c r="C22" s="137"/>
+      <c r="D22" s="137"/>
+      <c r="E22" s="137"/>
+      <c r="F22" s="316"/>
+      <c r="G22" s="143"/>
       <c r="H22" s="144"/>
       <c r="I22" s="114"/>
       <c r="J22" s="114"/>
@@ -10833,21 +9915,13 @@
       <c r="AA22" s="145"/>
     </row>
     <row r="23" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A23" s="956"/>
-      <c r="B23" s="1048">
-        <v>5</v>
-      </c>
-      <c r="C23" s="929" t="s">
-        <v>397</v>
-      </c>
-      <c r="D23" s="927" t="s">
-        <v>398</v>
-      </c>
-      <c r="E23" s="927"/>
-      <c r="F23" s="930" t="s">
-        <v>51</v>
-      </c>
-      <c r="G23" s="977"/>
+      <c r="A23" s="370"/>
+      <c r="B23" s="114"/>
+      <c r="C23" s="146"/>
+      <c r="D23" s="147"/>
+      <c r="E23" s="147"/>
+      <c r="F23" s="316"/>
+      <c r="G23" s="138"/>
       <c r="H23" s="144"/>
       <c r="I23" s="114"/>
       <c r="J23" s="114"/>
@@ -10873,15 +9947,15 @@
       <c r="AA23" s="145"/>
     </row>
     <row r="24" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A24" s="925"/>
-      <c r="B24" s="931">
+      <c r="A24" s="370"/>
+      <c r="B24" s="114">
         <v>6</v>
       </c>
-      <c r="C24" s="988"/>
-      <c r="D24" s="1078"/>
-      <c r="E24" s="991"/>
-      <c r="F24" s="997"/>
-      <c r="G24" s="1028"/>
+      <c r="C24" s="148"/>
+      <c r="D24" s="104"/>
+      <c r="E24" s="104"/>
+      <c r="F24" s="149"/>
+      <c r="G24" s="150"/>
       <c r="H24" s="144"/>
       <c r="I24" s="114"/>
       <c r="J24" s="114"/>
@@ -10907,15 +9981,15 @@
       <c r="AA24" s="145"/>
     </row>
     <row r="25" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A25" s="948"/>
-      <c r="B25" s="949">
+      <c r="A25" s="370"/>
+      <c r="B25" s="114">
         <v>7</v>
       </c>
-      <c r="C25" s="964"/>
-      <c r="D25" s="1043"/>
-      <c r="E25" s="946"/>
-      <c r="F25" s="1052"/>
-      <c r="G25" s="943"/>
+      <c r="C25" s="148"/>
+      <c r="D25" s="104"/>
+      <c r="E25" s="104"/>
+      <c r="F25" s="149"/>
+      <c r="G25" s="151"/>
       <c r="H25" s="144"/>
       <c r="I25" s="114"/>
       <c r="J25" s="114"/>
@@ -10941,15 +10015,15 @@
       <c r="AA25" s="145"/>
     </row>
     <row r="26" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A26" s="957"/>
-      <c r="B26" s="973">
+      <c r="A26" s="370"/>
+      <c r="B26" s="114">
         <v>8</v>
       </c>
-      <c r="C26" s="1051"/>
-      <c r="D26" s="954"/>
-      <c r="E26" s="1041"/>
-      <c r="F26" s="1015"/>
-      <c r="G26" s="951"/>
+      <c r="C26" s="148"/>
+      <c r="D26" s="104"/>
+      <c r="E26" s="104"/>
+      <c r="F26" s="149"/>
+      <c r="G26" s="152"/>
       <c r="H26" s="144"/>
       <c r="I26" s="114"/>
       <c r="J26" s="114"/>
@@ -10975,15 +10049,15 @@
       <c r="AA26" s="145"/>
     </row>
     <row r="27" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A27" s="1021"/>
-      <c r="B27" s="959">
+      <c r="A27" s="370"/>
+      <c r="B27" s="114">
         <v>9</v>
       </c>
-      <c r="C27" s="1065"/>
-      <c r="D27" s="1059"/>
-      <c r="E27" s="1014"/>
-      <c r="F27" s="1016"/>
-      <c r="G27" s="951"/>
+      <c r="C27" s="148"/>
+      <c r="D27" s="104"/>
+      <c r="E27" s="104"/>
+      <c r="F27" s="149"/>
+      <c r="G27" s="152"/>
       <c r="H27" s="153"/>
       <c r="I27" s="154"/>
       <c r="J27" s="154"/>
@@ -11009,15 +10083,15 @@
       <c r="AA27" s="145"/>
     </row>
     <row r="28" spans="1:27" ht="29.4" customHeight="1">
-      <c r="A28" s="1032"/>
-      <c r="B28" s="1035">
+      <c r="A28" s="405"/>
+      <c r="B28" s="116">
         <v>10</v>
       </c>
-      <c r="C28" s="987"/>
-      <c r="D28" s="966"/>
-      <c r="E28" s="966"/>
-      <c r="F28" s="994"/>
-      <c r="G28" s="971"/>
+      <c r="C28" s="159"/>
+      <c r="D28" s="160"/>
+      <c r="E28" s="160"/>
+      <c r="F28" s="161"/>
+      <c r="G28" s="162"/>
       <c r="H28" s="163"/>
       <c r="I28" s="116"/>
       <c r="J28" s="116"/>
@@ -11043,20 +10117,17 @@
       <c r="AA28" s="145"/>
     </row>
     <row r="29" spans="1:27" ht="27.45" customHeight="1">
-      <c r="A29" s="1067" t="s">
+      <c r="A29" s="395" t="s">
         <v>75</v>
       </c>
-      <c r="B29" s="1034"/>
-      <c r="C29" s="1062"/>
-      <c r="D29" s="960"/>
-      <c r="E29" s="960"/>
-      <c r="F29" s="1055" t="s">
+      <c r="B29" s="396"/>
+      <c r="C29" s="396"/>
+      <c r="D29" s="168"/>
+      <c r="E29" s="168"/>
+      <c r="F29" s="169" t="s">
         <v>76</v>
       </c>
-      <c r="G29" s="1017">
-        <f>M6*1.05</f>
-        <v>5250</v>
-      </c>
+      <c r="G29" s="170"/>
       <c r="H29" s="107"/>
       <c r="I29" s="107"/>
       <c r="J29" s="107"/>
@@ -11154,10 +10225,7 @@
       <c r="B39" s="174" t="s">
         <v>12</v>
       </c>
-      <c r="C39" s="175">
-        <f t="shared" ref="C39:C47" si="0">M6</f>
-        <v>5000</v>
-      </c>
+      <c r="C39" s="175"/>
       <c r="I39" s="402"/>
       <c r="J39" s="402"/>
       <c r="K39" s="402"/>
@@ -11172,10 +10240,7 @@
       <c r="B40" s="174" t="s">
         <v>18</v>
       </c>
-      <c r="C40" s="176">
-        <f t="shared" si="0"/>
-        <v>0.92</v>
-      </c>
+      <c r="C40" s="176"/>
       <c r="H40" s="109" t="s">
         <v>82</v>
       </c>
@@ -11193,10 +10258,7 @@
       <c r="B41" s="174" t="s">
         <v>18</v>
       </c>
-      <c r="C41" s="176">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
+      <c r="C41" s="176"/>
       <c r="I41" s="401"/>
       <c r="J41" s="401"/>
       <c r="K41" s="399"/>
@@ -11211,10 +10273,7 @@
       <c r="B42" s="174" t="s">
         <v>18</v>
       </c>
-      <c r="C42" s="175">
-        <f t="shared" si="0"/>
-        <v>4600</v>
-      </c>
+      <c r="C42" s="175"/>
       <c r="I42" s="401"/>
       <c r="J42" s="401"/>
       <c r="K42" s="399"/>
@@ -11229,10 +10288,7 @@
       <c r="B43" s="174" t="s">
         <v>25</v>
       </c>
-      <c r="C43" s="175">
-        <f t="shared" si="0"/>
-        <v>2</v>
-      </c>
+      <c r="C43" s="175"/>
       <c r="I43" s="401"/>
       <c r="J43" s="401"/>
       <c r="K43" s="399"/>
@@ -11247,10 +10303,7 @@
       <c r="B44" s="174" t="s">
         <v>18</v>
       </c>
-      <c r="C44" s="176">
-        <f t="shared" si="0"/>
-        <v>1.06</v>
-      </c>
+      <c r="C44" s="176"/>
       <c r="I44" s="401"/>
       <c r="J44" s="401"/>
       <c r="K44" s="399"/>
@@ -11265,10 +10318,7 @@
       <c r="B45" s="174" t="s">
         <v>18</v>
       </c>
-      <c r="C45" s="176">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="C45" s="176"/>
       <c r="I45" s="401"/>
       <c r="J45" s="401"/>
       <c r="K45" s="399"/>
@@ -11283,10 +10333,7 @@
       <c r="B46" s="174" t="s">
         <v>18</v>
       </c>
-      <c r="C46" s="176">
-        <f t="shared" si="0"/>
-        <v>1.02</v>
-      </c>
+      <c r="C46" s="176"/>
       <c r="I46" s="401"/>
       <c r="J46" s="401"/>
       <c r="K46" s="399"/>
@@ -11301,10 +10348,7 @@
       <c r="B47" s="174" t="s">
         <v>30</v>
       </c>
-      <c r="C47" s="177">
-        <f t="shared" si="0"/>
-        <v>4.1000000000000002E-2</v>
-      </c>
+      <c r="C47" s="177"/>
       <c r="I47" s="401"/>
       <c r="J47" s="401"/>
       <c r="K47" s="399"/>
@@ -12250,7 +11294,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0D00-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
     <pageSetUpPr fitToPage="1"/>
@@ -12338,15 +11382,12 @@
       <c r="A5" s="92" t="s">
         <v>116</v>
       </c>
-      <c r="C5" s="1121" t="str">
-        <f>In!C8</f>
-        <v>26BA2HKH00563000029</v>
-      </c>
-      <c r="D5" s="1094"/>
-      <c r="E5" s="1093"/>
-      <c r="F5" s="1113"/>
-      <c r="G5" s="1082"/>
-      <c r="H5" s="1083"/>
+      <c r="C5" s="575"/>
+      <c r="D5" s="575"/>
+      <c r="E5" s="93"/>
+      <c r="F5" s="93"/>
+      <c r="G5" s="93"/>
+      <c r="H5" s="93"/>
       <c r="I5" s="92" t="s">
         <v>3</v>
       </c>
@@ -12359,15 +11400,12 @@
       <c r="A6" s="92" t="s">
         <v>117</v>
       </c>
-      <c r="C6" s="1084" t="str">
-        <f>In!C7</f>
-        <v>BT1KH00563KP0004</v>
-      </c>
-      <c r="D6" s="1084"/>
-      <c r="E6" s="1084"/>
-      <c r="F6" s="1084"/>
-      <c r="G6" s="1084"/>
-      <c r="H6" s="1098"/>
+      <c r="C6" s="642"/>
+      <c r="D6" s="642"/>
+      <c r="E6" s="95"/>
+      <c r="F6" s="95"/>
+      <c r="G6" s="95"/>
+      <c r="H6" s="93"/>
       <c r="I6" s="92" t="s">
         <v>118</v>
       </c>
@@ -12379,15 +11417,12 @@
       <c r="A7" s="92" t="s">
         <v>120</v>
       </c>
-      <c r="C7" s="1117" t="str">
-        <f>In!C6</f>
-        <v>Bao giấy 25kg AM-20 Tân Châu</v>
-      </c>
-      <c r="D7" s="1105"/>
-      <c r="E7" s="1087"/>
-      <c r="F7" s="1120"/>
-      <c r="G7" s="1095"/>
-      <c r="H7" s="1085"/>
+      <c r="C7" s="575"/>
+      <c r="D7" s="575"/>
+      <c r="E7" s="575"/>
+      <c r="F7" s="575"/>
+      <c r="G7" s="575"/>
+      <c r="H7" s="575"/>
       <c r="I7" s="92" t="s">
         <v>121</v>
       </c>
@@ -12400,15 +11435,12 @@
         <v>123</v>
       </c>
       <c r="B8" s="94"/>
-      <c r="C8" s="1108" t="str">
-        <f>In!C5</f>
-        <v xml:space="preserve">NHÀ MÁY SX TINH BỘT SẮN TÂN CHÂU-CN CÔNG TY CPNS THỰC PHẨM QUẢNG NGÃI					</v>
-      </c>
-      <c r="D8" s="1119"/>
-      <c r="E8" s="1086"/>
-      <c r="F8" s="1081"/>
-      <c r="G8" s="1109"/>
-      <c r="H8" s="1088"/>
+      <c r="C8" s="575"/>
+      <c r="D8" s="575"/>
+      <c r="E8" s="575"/>
+      <c r="F8" s="575"/>
+      <c r="G8" s="575"/>
+      <c r="H8" s="575"/>
       <c r="I8" s="92" t="s">
         <v>124</v>
       </c>
@@ -12531,14 +11563,11 @@
         <v>135</v>
       </c>
       <c r="B16" s="653"/>
-      <c r="C16" s="1097" t="str">
-        <f>'In 1'!C16</f>
-        <v>Bao KP</v>
-      </c>
-      <c r="D16" s="1106"/>
-      <c r="E16" s="1089"/>
-      <c r="F16" s="1096"/>
-      <c r="G16" s="1090"/>
+      <c r="C16" s="441"/>
+      <c r="D16" s="441"/>
+      <c r="E16" s="441"/>
+      <c r="F16" s="441"/>
+      <c r="G16" s="453"/>
       <c r="I16" s="643" t="s">
         <v>137</v>
       </c>
@@ -12553,16 +11582,13 @@
         <v>139</v>
       </c>
       <c r="B17" s="653"/>
-      <c r="C17" s="1110" t="str">
-        <f>'In 1'!C17</f>
-        <v>500 x 920</v>
-      </c>
-      <c r="D17" s="1112"/>
-      <c r="E17" s="1091"/>
-      <c r="F17" s="1111" t="s">
+      <c r="C17" s="654"/>
+      <c r="D17" s="654"/>
+      <c r="E17" s="654"/>
+      <c r="F17" s="371" t="s">
         <v>140</v>
       </c>
-      <c r="G17" s="1092"/>
+      <c r="G17" s="646"/>
       <c r="I17" s="612"/>
       <c r="J17" s="613"/>
       <c r="K17" s="615"/>
@@ -12573,16 +11599,13 @@
         <v>141</v>
       </c>
       <c r="B18" s="653"/>
-      <c r="C18" s="1099" t="str">
-        <f>'In 1'!C18</f>
-        <v>500 x 920</v>
-      </c>
-      <c r="D18" s="1118"/>
-      <c r="E18" s="1104"/>
-      <c r="F18" s="1114" t="s">
+      <c r="C18" s="654"/>
+      <c r="D18" s="654"/>
+      <c r="E18" s="654"/>
+      <c r="F18" s="371" t="s">
         <v>140</v>
       </c>
-      <c r="G18" s="1122"/>
+      <c r="G18" s="646"/>
       <c r="I18" s="612"/>
       <c r="J18" s="613"/>
       <c r="K18" s="615"/>
@@ -12593,16 +11616,13 @@
         <v>142</v>
       </c>
       <c r="B19" s="653"/>
-      <c r="C19" s="1123">
-        <f>In!M6</f>
-        <v>5000</v>
-      </c>
-      <c r="D19" s="1116"/>
-      <c r="E19" s="1080"/>
-      <c r="F19" s="1115" t="s">
+      <c r="C19" s="654"/>
+      <c r="D19" s="654"/>
+      <c r="E19" s="654"/>
+      <c r="F19" s="371" t="s">
         <v>12</v>
       </c>
-      <c r="G19" s="1107"/>
+      <c r="G19" s="646"/>
       <c r="I19" s="612"/>
       <c r="J19" s="613"/>
       <c r="K19" s="615"/>
@@ -12613,16 +11633,13 @@
         <v>143</v>
       </c>
       <c r="B20" s="656"/>
-      <c r="C20" s="1101">
-        <f>C19</f>
-        <v>5000</v>
-      </c>
-      <c r="D20" s="1100"/>
-      <c r="E20" s="1102"/>
-      <c r="F20" s="1103" t="s">
+      <c r="C20" s="657"/>
+      <c r="D20" s="657"/>
+      <c r="E20" s="657"/>
+      <c r="F20" s="439" t="s">
         <v>12</v>
       </c>
-      <c r="G20" s="1079"/>
+      <c r="G20" s="658"/>
       <c r="I20" s="647"/>
       <c r="J20" s="648"/>
       <c r="K20" s="650"/>
@@ -17870,7 +16887,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-1100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
     <pageSetUpPr fitToPage="1"/>
@@ -17982,15 +16999,12 @@
         <v>116</v>
       </c>
       <c r="B5" s="767"/>
-      <c r="C5" s="1150" t="str">
-        <f>'In 2'!C5</f>
-        <v>26BA2HKH00563000029</v>
-      </c>
-      <c r="D5" s="1136"/>
-      <c r="E5" s="1135"/>
-      <c r="F5" s="1146"/>
-      <c r="G5" s="1125"/>
-      <c r="H5" s="1126"/>
+      <c r="C5" s="768"/>
+      <c r="D5" s="768"/>
+      <c r="E5" s="768"/>
+      <c r="F5" s="768"/>
+      <c r="G5" s="768"/>
+      <c r="H5" s="768"/>
       <c r="I5" s="48" t="s">
         <v>3</v>
       </c>
@@ -18025,15 +17039,12 @@
         <v>117</v>
       </c>
       <c r="B6" s="769"/>
-      <c r="C6" s="1127" t="str">
-        <f>'In 2'!C6</f>
-        <v>BT1KH00563KP0004</v>
-      </c>
-      <c r="D6" s="1137"/>
-      <c r="E6" s="1128"/>
-      <c r="F6" s="1151"/>
-      <c r="G6" s="1129"/>
-      <c r="H6" s="1140"/>
+      <c r="C6" s="770"/>
+      <c r="D6" s="770"/>
+      <c r="E6" s="770"/>
+      <c r="F6" s="770"/>
+      <c r="G6" s="770"/>
+      <c r="H6" s="770"/>
       <c r="I6" s="48" t="s">
         <v>184</v>
       </c>
@@ -18052,15 +17063,12 @@
         <v>120</v>
       </c>
       <c r="B7" s="769"/>
-      <c r="C7" s="1147" t="str">
-        <f>'In 2'!C7</f>
-        <v>Bao giấy 25kg AM-20 Tân Châu</v>
-      </c>
-      <c r="D7" s="1141"/>
-      <c r="E7" s="1132"/>
-      <c r="F7" s="1149"/>
-      <c r="G7" s="1138"/>
-      <c r="H7" s="1130"/>
+      <c r="C7" s="770"/>
+      <c r="D7" s="770"/>
+      <c r="E7" s="770"/>
+      <c r="F7" s="770"/>
+      <c r="G7" s="770"/>
+      <c r="H7" s="770"/>
       <c r="I7" s="5" t="s">
         <v>121</v>
       </c>
@@ -18080,15 +17088,12 @@
         <v>123</v>
       </c>
       <c r="B8" s="769"/>
-      <c r="C8" s="1143" t="str">
-        <f>'In 2'!C8</f>
-        <v xml:space="preserve">NHÀ MÁY SX TINH BỘT SẮN TÂN CHÂU-CN CÔNG TY CPNS THỰC PHẨM QUẢNG NGÃI					</v>
-      </c>
-      <c r="D8" s="1148"/>
-      <c r="E8" s="1131"/>
-      <c r="F8" s="1124"/>
-      <c r="G8" s="1145"/>
-      <c r="H8" s="1133"/>
+      <c r="C8" s="768"/>
+      <c r="D8" s="768"/>
+      <c r="E8" s="768"/>
+      <c r="F8" s="768"/>
+      <c r="G8" s="768"/>
+      <c r="H8" s="768"/>
       <c r="I8" s="5" t="s">
         <v>124</v>
       </c>
@@ -18260,20 +17265,14 @@
         <v>186</v>
       </c>
       <c r="B16" s="13"/>
-      <c r="C16" s="1139">
-        <f>'In 2'!C16</f>
-        <v>4600</v>
-      </c>
-      <c r="D16" s="1142"/>
+      <c r="C16" s="801"/>
+      <c r="D16" s="802"/>
       <c r="E16" s="803" t="s">
         <v>187</v>
       </c>
       <c r="F16" s="803"/>
-      <c r="G16" s="1134">
-        <f>Tráng!M9</f>
-        <v>4600</v>
-      </c>
-      <c r="H16" s="1144"/>
+      <c r="G16" s="804"/>
+      <c r="H16" s="805"/>
       <c r="I16" s="7"/>
       <c r="J16" s="806" t="s">
         <v>137</v>
@@ -22440,7 +21439,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-1300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <sheetPr>
     <tabColor rgb="FF00B0F0"/>
     <pageSetUpPr fitToPage="1"/>
@@ -22528,15 +21527,12 @@
         <v>116</v>
       </c>
       <c r="B5" s="576"/>
-      <c r="C5" s="1196" t="str">
-        <f>'In 2'!C5</f>
-        <v>26BA2HKH00563000029</v>
-      </c>
-      <c r="D5" s="1166"/>
-      <c r="E5" s="1165"/>
-      <c r="F5" s="1185"/>
-      <c r="G5" s="1155"/>
-      <c r="H5" s="1156"/>
+      <c r="C5" s="575"/>
+      <c r="D5" s="575"/>
+      <c r="E5" s="575"/>
+      <c r="F5" s="575"/>
+      <c r="G5" s="575"/>
+      <c r="H5" s="575"/>
       <c r="I5" s="92" t="s">
         <v>3</v>
       </c>
@@ -22563,15 +21559,12 @@
         <v>117</v>
       </c>
       <c r="B6" s="577"/>
-      <c r="C6" s="1157" t="str">
-        <f>'In 2'!C6</f>
-        <v>BT1KH00563KP0004</v>
-      </c>
-      <c r="D6" s="1167"/>
-      <c r="E6" s="1158"/>
-      <c r="F6" s="1199"/>
-      <c r="G6" s="1159"/>
-      <c r="H6" s="1169"/>
+      <c r="C6" s="338"/>
+      <c r="D6" s="338"/>
+      <c r="E6" s="338"/>
+      <c r="F6" s="338"/>
+      <c r="G6" s="338"/>
+      <c r="H6" s="338"/>
       <c r="I6" s="92" t="s">
         <v>184</v>
       </c>
@@ -22585,15 +21578,12 @@
         <v>120</v>
       </c>
       <c r="B7" s="577"/>
-      <c r="C7" s="1190" t="str">
-        <f>'In 2'!C7</f>
-        <v>Bao giấy 25kg AM-20 Tân Châu</v>
-      </c>
-      <c r="D7" s="1177"/>
-      <c r="E7" s="1162"/>
-      <c r="F7" s="1194"/>
-      <c r="G7" s="1168"/>
-      <c r="H7" s="1160"/>
+      <c r="C7" s="338"/>
+      <c r="D7" s="338"/>
+      <c r="E7" s="338"/>
+      <c r="F7" s="338"/>
+      <c r="G7" s="338"/>
+      <c r="H7" s="338"/>
       <c r="I7" s="180" t="s">
         <v>121</v>
       </c>
@@ -22607,15 +21597,12 @@
         <v>123</v>
       </c>
       <c r="B8" s="577"/>
-      <c r="C8" s="1180" t="str">
-        <f>'In 2'!C8</f>
-        <v xml:space="preserve">NHÀ MÁY SX TINH BỘT SẮN TÂN CHÂU-CN CÔNG TY CPNS THỰC PHẨM QUẢNG NGÃI					</v>
-      </c>
-      <c r="D8" s="1192"/>
-      <c r="E8" s="1161"/>
-      <c r="F8" s="1154"/>
-      <c r="G8" s="1182"/>
-      <c r="H8" s="1163"/>
+      <c r="C8" s="575"/>
+      <c r="D8" s="575"/>
+      <c r="E8" s="575"/>
+      <c r="F8" s="575"/>
+      <c r="G8" s="575"/>
+      <c r="H8" s="575"/>
       <c r="I8" s="180" t="s">
         <v>124</v>
       </c>
@@ -22627,9 +21614,9 @@
     <row r="9" spans="1:24" ht="15" customHeight="1">
       <c r="A9" s="94"/>
       <c r="B9" s="94"/>
-      <c r="C9" s="1183"/>
-      <c r="D9" s="1193"/>
-      <c r="E9" s="1179"/>
+      <c r="C9" s="94"/>
+      <c r="D9" s="94"/>
+      <c r="E9" s="94"/>
       <c r="I9" s="94"/>
       <c r="K9" s="94"/>
     </row>
@@ -22735,10 +21722,7 @@
       </c>
       <c r="B16" s="653"/>
       <c r="C16" s="653"/>
-      <c r="D16" s="897">
-        <f>G18+G19</f>
-        <v>15.244399999999999</v>
-      </c>
+      <c r="D16" s="897"/>
       <c r="E16" s="898"/>
       <c r="F16" s="333" t="s">
         <v>51</v>
@@ -22785,26 +21769,13 @@
       <c r="A18" s="140">
         <v>1</v>
       </c>
-      <c r="B18" s="1184">
-        <f>Dán!C17</f>
-        <v>9415</v>
-      </c>
-      <c r="C18" s="1170"/>
-      <c r="D18" s="1191" t="str">
-        <f>Dán!D17</f>
-        <v>NHPPFC9415G01</v>
-      </c>
-      <c r="E18" s="1176">
-        <v>0.6</v>
-      </c>
-      <c r="F18" s="1186" t="s">
-        <v>51</v>
-      </c>
-      <c r="G18" s="1197">
-        <f>Dán!G17</f>
-        <v>9.1466399999999997</v>
-      </c>
-      <c r="H18" s="1187"/>
+      <c r="B18" s="333"/>
+      <c r="C18" s="333"/>
+      <c r="D18" s="210"/>
+      <c r="E18" s="188"/>
+      <c r="F18" s="189"/>
+      <c r="G18" s="189"/>
+      <c r="H18" s="186"/>
       <c r="J18" s="672"/>
       <c r="K18" s="673"/>
       <c r="L18" s="191"/>
@@ -22814,44 +21785,25 @@
       <c r="A19" s="140">
         <v>2</v>
       </c>
-      <c r="B19" s="1174" t="str">
-        <f>Dán!C18</f>
-        <v>Vistamaxx</v>
-      </c>
-      <c r="C19" s="1198"/>
-      <c r="D19" s="1189" t="str">
-        <f>Dán!D18</f>
-        <v>NHVITAMAX0001</v>
-      </c>
-      <c r="E19" s="1153">
-        <v>0.4</v>
-      </c>
-      <c r="F19" s="1188" t="s">
-        <v>51</v>
-      </c>
-      <c r="G19" s="1178">
-        <f>Dán!G18</f>
-        <v>6.0977600000000001</v>
-      </c>
-      <c r="H19" s="1195"/>
+      <c r="B19" s="333"/>
+      <c r="C19" s="333"/>
+      <c r="D19" s="210"/>
+      <c r="E19" s="188"/>
+      <c r="F19" s="189"/>
+      <c r="G19" s="189"/>
+      <c r="H19" s="190"/>
     </row>
     <row r="20" spans="1:14" ht="18" customHeight="1">
       <c r="A20" s="140">
         <v>3</v>
       </c>
-      <c r="B20" s="1181" t="str">
-        <f>Dán!C19</f>
-        <v>Keo Acrylic</v>
-      </c>
-      <c r="C20" s="1172"/>
-      <c r="D20" s="1171" t="str">
-        <f>Dán!D19</f>
-        <v>PKACRYLIC0001</v>
-      </c>
-      <c r="E20" s="1173"/>
-      <c r="F20" s="1175"/>
-      <c r="G20" s="1152"/>
-      <c r="H20" s="1164"/>
+      <c r="B20" s="441"/>
+      <c r="C20" s="441"/>
+      <c r="D20" s="210"/>
+      <c r="E20" s="188"/>
+      <c r="F20" s="114"/>
+      <c r="G20" s="189"/>
+      <c r="H20" s="190"/>
       <c r="J20" s="348" t="s">
         <v>192</v>
       </c>

</xml_diff>